<commit_message>
Modèle BLI : colonne N° BDS plus large pour plusieurs N° sur une ligne
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KktRdaesqzLGGy7kb2yhrm
</commit_message>
<xml_diff>
--- a/modeles/Modele_BLI_numerique.xlsx
+++ b/modeles/Modele_BLI_numerique.xlsx
@@ -999,11 +999,11 @@
   <dimension ref="A1:G108"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
   </cols>

</xml_diff>